<commit_message>
Add AdLabs audit skill + /adlabs-audit; align audit skills on shared playbook; public-safe genericization
- New amazon-adlabs-audit skill + /adlabs-audit command (MCP-native audit for managed AdLabs clients; context-first, Optimization-Group grading, Rank-Radar verification, phased-transition posture, read-only)

- amazon-ad-audit skill/toolkit + playbook now the shared narrative/design source of truth; routing in agent.md/AGENTS.md

- docs/public-release-checklist.md (agent-neutral pre-push checklist)

- Also includes in-progress amazon-campaign-builder + seo/flatfilepro updates

- Genericized client/prospect names across tracked files for public-safe release; client config JSONs remain gitignored

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/amazon-seo-keyword-workbook/template_keyword_workbook.xlsx
+++ b/tools/amazon-seo-keyword-workbook/template_keyword_workbook.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="ASINs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="1. Root Keywords" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2.1 MKL DataDive 1%" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2.2 Never KWs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="3.1 MKL DataDive 30%" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="3.2 Outlier KWs" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="4. SEO Text" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="5. Campaign Structure" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="POE Raw - Products" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="POE Raw - Search Terms" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="POE Raw - Reviews" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="POE Raw - Returns" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="POE Raw - Related Niches" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="POE Semantic Insights" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ASINs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. Root Keywords" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.1 MKL DataDive 1%" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.2 Never KWs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.1 MKL DataDive 30%" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.2 Outlier KWs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. SEO Text" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. Campaign Structure" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POE Raw - Products" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POE Raw - Search Terms" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POE Raw - Reviews" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POE Raw - Returns" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POE Raw - Related Niches" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POE Semantic Insights" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1. Root Keywords'!$A$1:$D$45</definedName>
@@ -169,7 +169,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border/>
     <border>
       <bottom style="thin">
@@ -259,11 +259,25 @@
         <color rgb="FF000000"/>
       </top>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -444,6 +458,15 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -13147,78 +13170,89 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col width="23.38" customWidth="1" style="53" min="1" max="1"/>
-    <col width="72.38" customWidth="1" style="53" min="2" max="3"/>
-    <col width="12.63" customWidth="1" style="53" min="4" max="6"/>
+    <col width="26" customWidth="1" style="53" min="1" max="1"/>
+    <col width="60" customWidth="1" style="53" min="2" max="3"/>
+    <col width="60" customWidth="1" style="53" min="3" max="3"/>
+    <col width="50" customWidth="1" style="53" min="4" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1" s="53">
-      <c r="A1" s="13" t="n"/>
-      <c r="B1" s="59" t="inlineStr">
+      <c r="A1" s="71" t="n"/>
+      <c r="B1" s="72" t="inlineStr">
         <is>
           <t>Old Listing</t>
         </is>
       </c>
-      <c r="C1" s="60" t="inlineStr">
+      <c r="C1" s="72" t="inlineStr">
         <is>
           <t>New Listing</t>
         </is>
       </c>
-      <c r="D1" s="16" t="inlineStr">
+      <c r="D1" s="71" t="inlineStr">
         <is>
           <t>Session ID</t>
         </is>
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1" s="53">
-      <c r="A2" s="17" t="n"/>
-      <c r="B2" s="61" t="n"/>
-      <c r="C2" s="62" t="n"/>
+      <c r="A2" s="71" t="n"/>
+      <c r="B2" s="73" t="n"/>
+      <c r="C2" s="73" t="n"/>
+      <c r="D2" s="73" t="n"/>
     </row>
     <row r="3" ht="15.75" customHeight="1" s="53">
-      <c r="A3" s="13" t="n"/>
-      <c r="B3" s="63" t="n"/>
-      <c r="C3" s="64" t="n"/>
+      <c r="A3" s="71" t="n"/>
+      <c r="B3" s="73" t="n"/>
+      <c r="C3" s="73" t="n"/>
+      <c r="D3" s="73" t="n"/>
     </row>
     <row r="4" ht="15.75" customHeight="1" s="53">
-      <c r="A4" s="22" t="n"/>
-      <c r="B4" s="65" t="n"/>
-      <c r="C4" s="66" t="n"/>
+      <c r="A4" s="71" t="n"/>
+      <c r="B4" s="73" t="n"/>
+      <c r="C4" s="73" t="n"/>
+      <c r="D4" s="73" t="n"/>
     </row>
     <row r="5" ht="15.75" customHeight="1" s="53">
-      <c r="A5" s="22" t="n"/>
-      <c r="B5" s="65" t="n"/>
-      <c r="C5" s="66" t="n"/>
+      <c r="A5" s="71" t="n"/>
+      <c r="B5" s="73" t="n"/>
+      <c r="C5" s="73" t="n"/>
+      <c r="D5" s="73" t="n"/>
     </row>
     <row r="6" ht="15.75" customHeight="1" s="53">
-      <c r="A6" s="22" t="n"/>
-      <c r="B6" s="65" t="n"/>
-      <c r="C6" s="66" t="n"/>
+      <c r="A6" s="71" t="n"/>
+      <c r="B6" s="73" t="n"/>
+      <c r="C6" s="73" t="n"/>
+      <c r="D6" s="73" t="n"/>
     </row>
     <row r="7" ht="15.75" customHeight="1" s="53">
-      <c r="A7" s="22" t="n"/>
-      <c r="B7" s="65" t="n"/>
-      <c r="C7" s="66" t="n"/>
+      <c r="A7" s="71" t="n"/>
+      <c r="B7" s="73" t="n"/>
+      <c r="C7" s="73" t="n"/>
+      <c r="D7" s="73" t="n"/>
     </row>
     <row r="8" ht="15.75" customHeight="1" s="53">
-      <c r="A8" s="25" t="n"/>
-      <c r="B8" s="67" t="n"/>
-      <c r="C8" s="68" t="n"/>
+      <c r="A8" s="71" t="n"/>
+      <c r="B8" s="73" t="n"/>
+      <c r="C8" s="73" t="n"/>
+      <c r="D8" s="73" t="n"/>
     </row>
     <row r="9" ht="15.75" customHeight="1" s="53">
-      <c r="A9" s="28" t="n"/>
-      <c r="B9" s="65" t="n"/>
-      <c r="C9" s="66" t="n"/>
+      <c r="A9" s="71" t="n"/>
+      <c r="B9" s="73" t="n"/>
+      <c r="C9" s="73" t="n"/>
+      <c r="D9" s="73" t="n"/>
     </row>
     <row r="10" ht="15.75" customHeight="1" s="53">
-      <c r="A10" s="29" t="n"/>
-      <c r="B10" s="65" t="n"/>
-      <c r="C10" s="66" t="n"/>
+      <c r="A10" s="71" t="n"/>
+      <c r="B10" s="73" t="n"/>
+      <c r="C10" s="73" t="n"/>
+      <c r="D10" s="73" t="n"/>
     </row>
     <row r="11" ht="15.75" customHeight="1" s="53">
-      <c r="A11" s="30" t="n"/>
-      <c r="B11" s="67" t="n"/>
-      <c r="C11" s="69" t="n"/>
+      <c r="A11" s="71" t="n"/>
+      <c r="B11" s="73" t="n"/>
+      <c r="C11" s="73" t="n"/>
+      <c r="D11" s="73" t="n"/>
     </row>
     <row r="12" ht="15.75" customHeight="1" s="53"/>
     <row r="13" ht="15.75" customHeight="1" s="53"/>

</xml_diff>